<commit_message>
data(personal): publish administrative-division workbook
</commit_message>
<xml_diff>
--- a/docs/personal/administrative-divisions/data/administrative-divisions-indonesia.xlsx
+++ b/docs/personal/administrative-divisions/data/administrative-divisions-indonesia.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Data" sheetId="1" r:id="R330e0da2ae2c439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Info" sheetId="2" r:id="Rf0042d9b6203410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Data" sheetId="1" r:id="R3437e9d553ec4e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Info" sheetId="2" r:id="Rb66e326acd1548c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -110,8 +110,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AdministrativeDivisionsTable" displayName="AdministrativeDivisionsTable" ref="A1:G53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G53"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AdministrativeDivisionsTable" displayName="AdministrativeDivisionsTable" ref="A1:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G55"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="code"/>
     <x:tableColumn id="2" name="parent_code"/>
@@ -1344,7 +1344,7 @@
         <x:v>ID-BB-BTM</x:v>
       </x:c>
       <x:c r="B45" s="10" t="str">
-        <x:v>ID-BB</x:v>
+        <x:v>ID-KR</x:v>
       </x:c>
       <x:c r="C45" s="11" t="n">
         <x:v>3</x:v>
@@ -1546,10 +1546,56 @@
         <x:v>active</x:v>
       </x:c>
     </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>ID-LA</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="C54" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>楠榜省</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>Lampung</x:v>
+      </x:c>
+      <x:c r="F54" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>ID-KR</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="C55" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>廖内群岛省</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>Riau Islands</x:v>
+      </x:c>
+      <x:c r="F55" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e6f0be95d0a4f38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc06fd74efe194e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1591,7 +1637,23 @@
         <x:v>note</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>Generated from the project administrative-division source workbook.</x:v>
+        <x:v>Corrected 2026-10-18: add Lampung and Riau Islands; move Batam to Riau Islands while retaining its existing stable code.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>province_source</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>https://sirusa.web.bps.go.id/metadata/variabel/de34ad05-08e6-9650-1f6c-5acc7f3eafe8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>batam_source</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>https://batamkota.bps.go.id/id</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>